<commit_message>
Fix export alignment and refresh docs notebook workflow
</commit_message>
<xml_diff>
--- a/mario/test/supporting_files/cvxlab/mario_add_sector_split/input_data/input_data.xlsx
+++ b/mario/test/supporting_files/cvxlab/mario_add_sector_split/input_data/input_data.xlsx
@@ -9,13 +9,14 @@
   <sheets>
     <sheet name="Zold" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Yold" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Xnew" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="VA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Vold" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="V0" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Trade" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Znew0" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Trade_selector" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="I_p_pn" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="tol" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Z0" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="X" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Trade_selector" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="I_p_pn" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="tol" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -480,6 +481,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F2" t="n">
+        <v>5357798.997117119</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -505,6 +509,9 @@
           <t>Agriculture</t>
         </is>
       </c>
+      <c r="F3" t="n">
+        <v>1122396.507146856</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -530,6 +537,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F4" t="n">
+        <v>22892840.59900518</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -555,6 +565,9 @@
           <t>New services</t>
         </is>
       </c>
+      <c r="F5" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -580,6 +593,9 @@
           <t>Services</t>
         </is>
       </c>
+      <c r="F6" t="n">
+        <v>10650955.19256881</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -605,6 +621,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -630,6 +649,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F8" t="n">
+        <v>9737508.813505344</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -655,6 +677,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F9" t="n">
+        <v>50607.80686140568</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -680,6 +705,9 @@
           <t>Agriculture</t>
         </is>
       </c>
+      <c r="F10" t="n">
+        <v>1413.697219031487</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -705,6 +733,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F11" t="n">
+        <v>134910.6575432917</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -730,6 +761,9 @@
           <t>New services</t>
         </is>
       </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -755,6 +789,9 @@
           <t>Services</t>
         </is>
       </c>
+      <c r="F13" t="n">
+        <v>30367.20970916997</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -780,6 +817,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -805,6 +845,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F15" t="n">
+        <v>27813.85721607183</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -830,6 +873,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F16" t="n">
+        <v>2596.040895054911</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -855,6 +901,9 @@
           <t>Agriculture</t>
         </is>
       </c>
+      <c r="F17" t="n">
+        <v>6890.986703343548</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -880,6 +929,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F18" t="n">
+        <v>133519.3206683478</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -905,6 +957,9 @@
           <t>New services</t>
         </is>
       </c>
+      <c r="F19" t="n">
+        <v>525</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -930,6 +985,9 @@
           <t>Services</t>
         </is>
       </c>
+      <c r="F20" t="n">
+        <v>65558.29153130467</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -955,6 +1013,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -980,6 +1041,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F22" t="n">
+        <v>15550.45492095414</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1005,6 +1069,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F23" t="n">
+        <v>30635.04569590089</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1030,6 +1097,9 @@
           <t>Agriculture</t>
         </is>
       </c>
+      <c r="F24" t="n">
+        <v>9736.931971973165</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1055,6 +1125,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F25" t="n">
+        <v>287300.6733546407</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1080,6 +1153,9 @@
           <t>New services</t>
         </is>
       </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1105,6 +1181,9 @@
           <t>Services</t>
         </is>
       </c>
+      <c r="F27" t="n">
+        <v>161126.9406138842</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1130,6 +1209,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1154,6 +1236,66 @@
         <is>
           <t>Industry</t>
         </is>
+      </c>
+      <c r="F29" t="n">
+        <v>312355.7752418953</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>scalar_Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>values</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>delta</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1226,6 +1368,9 @@
           <t>Final demand</t>
         </is>
       </c>
+      <c r="F2" t="n">
+        <v>18160868.99186129</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1251,6 +1396,9 @@
           <t>Final demand</t>
         </is>
       </c>
+      <c r="F3" t="n">
+        <v>121750.6625725599</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1276,6 +1424,9 @@
           <t>Final demand</t>
         </is>
       </c>
+      <c r="F4" t="n">
+        <v>231650.9630397502</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1300,6 +1451,9 @@
         <is>
           <t>Final demand</t>
         </is>
+      </c>
+      <c r="F5" t="n">
+        <v>299898.9111312811</v>
       </c>
     </row>
   </sheetData>
@@ -1313,7 +1467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1324,15 +1478,20 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>region_from_Name</t>
+          <t>factor_Name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>sector_from_Name</t>
+          <t>region_to_Name</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
+        <is>
+          <t>sector_to_Name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
         <is>
           <t>values</t>
         </is>
@@ -1344,13 +1503,21 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Reg1</t>
+          <t>Capital</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Industry</t>
-        </is>
+          <t>Reg1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>5616640.677690812</v>
       </c>
     </row>
     <row r="3">
@@ -1359,13 +1526,21 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Reg1</t>
+          <t>Capital</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>New industry</t>
-        </is>
+          <t>Reg2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>101949.2414284951</v>
       </c>
     </row>
     <row r="4">
@@ -1374,13 +1549,21 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Reg2</t>
+          <t>Taxes</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Industry</t>
-        </is>
+          <t>Reg1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>3047095.547721097</v>
       </c>
     </row>
     <row r="5">
@@ -1389,13 +1572,67 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Reg2</t>
+          <t>Taxes</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>New industry</t>
-        </is>
+          <t>Reg2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>36852.4819132207</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Wages</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Reg1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>6311953.060686084</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Wages</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Reg2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>213257.4792719122</v>
       </c>
     </row>
   </sheetData>
@@ -1409,7 +1646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1420,15 +1657,20 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>factor_Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>region_to_Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>sector_to_Name</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>values</t>
         </is>
@@ -1440,13 +1682,21 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Reg1</t>
+          <t>Capital</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>New industry</t>
-        </is>
+          <t>Reg1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>5236405.671792497</v>
       </c>
     </row>
     <row r="3">
@@ -1455,13 +1705,251 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Reg2</t>
+          <t>Capital</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>New industry</t>
-        </is>
+          <t>Reg1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>380325.4886939208</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Capital</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Reg2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>54154.61845469403</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Capital</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Reg2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>47856.21566152293</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Taxes</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Reg1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>2856981.891385896</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Taxes</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Reg1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>190162.7443469604</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Taxes</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Reg2</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>12946.63852875086</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Taxes</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Reg2</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>23928.10783076147</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Wages</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Reg1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>5931729.256111095</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Wages</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Reg1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>380325.4886939208</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Wages</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Reg2</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>165530.1032284296</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Wages</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Reg2</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>47856.21566152293</v>
       </c>
     </row>
   </sheetData>
@@ -1524,6 +2012,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1544,6 +2035,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="E3" t="n">
+        <v>98591.98503</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1564,6 +2058,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="E4" t="n">
+        <v>980167.8945000001</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1583,6 +2080,9 @@
         <is>
           <t>New industry</t>
         </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1655,6 +2155,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F2" t="n">
+        <v>3457178.825293626</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1680,6 +2183,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F3" t="n">
+        <v>1900706.484738877</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1705,6 +2211,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F4" t="n">
+        <v>2377034.304337005</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1730,6 +2239,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1755,6 +2267,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1780,6 +2295,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1805,6 +2323,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F8" t="n">
+        <v>5940474.774304985</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1830,6 +2351,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F9" t="n">
+        <v>3797190.908238319</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1855,6 +2379,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1880,6 +2407,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F11" t="n">
+        <v>149052.9962379021</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1905,6 +2435,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F12" t="n">
+        <v>299101.3478845183</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1930,6 +2463,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1955,6 +2491,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1980,6 +2519,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2005,6 +2547,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2030,6 +2575,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F17" t="n">
+        <v>39129.4760703136</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2055,6 +2603,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F18" t="n">
+        <v>1675.123985951943</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2080,6 +2631,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F19" t="n">
+        <v>920.9587307275248</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -2105,6 +2659,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F20" t="n">
+        <v>475406.8608674011</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2130,6 +2687,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2155,6 +2715,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2180,6 +2743,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2205,6 +2771,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F24" t="n">
+        <v>9486.726734334083</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2230,6 +2799,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F25" t="n">
+        <v>6063.978700889161</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2255,6 +2827,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2280,6 +2855,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F27" t="n">
+        <v>90228.08206971256</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2305,6 +2883,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F28" t="n">
+        <v>59820.26957690367</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2330,6 +2911,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2355,6 +2939,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2380,6 +2967,9 @@
           <t>New industry</t>
         </is>
       </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2405,6 +2995,9 @@
           <t>Industry</t>
         </is>
       </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2429,6 +3022,9 @@
         <is>
           <t>New industry</t>
         </is>
+      </c>
+      <c r="F33" t="n">
+        <v>439432.6805449158</v>
       </c>
     </row>
   </sheetData>
@@ -2442,7 +3038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2453,20 +3049,15 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>region_from_Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>sector_from_Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>region_from_Name</t>
-        </is>
-      </c>
       <c r="D1" t="inlineStr">
-        <is>
-          <t>region_to_Name</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
         <is>
           <t>values</t>
         </is>
@@ -2478,18 +3069,16 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>New industry</t>
+          <t>Reg1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Reg1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Reg1</t>
-        </is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>43608221.97888111</v>
       </c>
     </row>
     <row r="3">
@@ -2498,18 +3087,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>New industry</t>
+          <t>Reg1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Reg1</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Reg2</t>
-        </is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>9508137.217348021</v>
       </c>
     </row>
     <row r="4">
@@ -2518,18 +3105,16 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>New industry</t>
+          <t>Reg2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Reg2</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Reg1</t>
-        </is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -2538,18 +3123,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>New industry</t>
+          <t>Reg2</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Reg2</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Reg2</t>
-        </is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1196405.391538073</v>
       </c>
     </row>
   </sheetData>
@@ -2563,7 +3146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2574,15 +3157,20 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>sector_to_Name</t>
+          <t>sector_from_Name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>sector_from_Name</t>
+          <t>region_from_Name</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
+        <is>
+          <t>region_to_Name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
         <is>
           <t>values</t>
         </is>
@@ -2594,13 +3182,21 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>New industry</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Industry</t>
-        </is>
+          <t>Reg1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Reg1</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -2609,13 +3205,67 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>New industry</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>New industry</t>
-        </is>
+          <t>Reg1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Reg2</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Reg2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Reg1</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Reg2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Reg2</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2629,7 +3279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2640,10 +3290,15 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>scalar_Name</t>
+          <t>sector_to_Name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
+        <is>
+          <t>sector_from_Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
         <is>
           <t>values</t>
         </is>
@@ -2655,10 +3310,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>delta</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -2666,10 +3328,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>eps</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>